<commit_message>
Regenerate FC findings cache with today's resolver/rule fixes
Reflects the corrected resolver (cash-flow not presented, share-based false) and
3.16B rejection. The big false positives Phil flagged are gone (consolidation,
5.7E, going-concern verify). However the disclosure findings still carry
rule-quality noise (6.2 duplicated, 9.8 mis-gated consolidation rule, 3.6
departure, 3.21/3.17 complete-set) — the same per-rule calibration the questions
needed, now on the findings side. Interview is clean (5 confirms); findings need
a rule-by-rule pass with Phil before they're demo-clean.
</commit_message>
<xml_diff>
--- a/build/summaries/FC-register.xlsx
+++ b/build/summaries/FC-register.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Questions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues register'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues register'!$A$1:$H$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,28 +511,28 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Required disclosures missing: 4</t>
+          <t>Required disclosures missing: 8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Disclosures to verify present: 3</t>
+          <t>Disclosures to verify present: 4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Numerical findings: 4 (2 could not be evaluated)</t>
+          <t>Numerical findings: 5 (2 could not be evaluated)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Open questions for the reviewer: 27</t>
+          <t>Open questions for the reviewer: 6</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Checklist outcomes: undetermined=77, not_applicable=210, encouraged=2, applicable=77</t>
+          <t>Checklist outcomes: not_applicable=284, encouraged=2, applicable=72, undetermined=7</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -628,12 +628,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - verify present</t>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>FRS102 5.7E</t>
+          <t>FRS102 3.6</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -643,12 +643,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Could not confirm this required disclosure - verify: Disclose on the face of the income statement (or statement of comprehensive income if presented) an amount comprising the total of [the items required by paragraph 5.7E — paragraph text as supplied is truncated and the specific sub-items cannot be determined from the verbatim text provided]</t>
+          <t>Required disclosure not found in the accounts: Where an entity departed from a requirement of FRS 102 or applicable legislation in a prior period and that departure affects amounts recognised in the current period, disclose the information required by paragraph 3.5(c).</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>The income statement shows turnover, cost of sales, gross profit, administrative expenses, operating (loss)/profit, interest, and tax. The specific sub-items required by paragraph 5.7E cannot be determined from the truncated paragraph text provided, making it impossible to verify compliance.</t>
+          <t>There is no disclosure of any prior period departure from FRS 102 or applicable legislation that affects amounts in the current period, beyond the restatement of group undertaking balances which is explained in note 14 but not framed as a departure from a requirement.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - MISSING</t>
+          <t>Disclosure - verify present</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>FRS102 6.2</t>
+          <t>FRS102 3.17</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -679,12 +679,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: the effects of changes in accounting policies and corrections of material errors recognised in the period (this row covers one sub-element of paragraph 6.2; companion rows should address profit or loss, OCI, and investments/dividends/distributions)</t>
+          <t>Could not confirm this required disclosure - verify: A complete set of financial statements shall include all of the required components as listed in paragraph 3.17 (e.g. a statement of financial position, a statement of comprehensive income or equivalent, a cash flow statement, a statement of changes in equity, and notes).</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>The statement of changes in equity shows only opening balances, profit/loss for the year, and closing balances. There is no row showing effects of changes in accounting policies or corrections of material errors (though a restatement of 2023 debtor/creditor balances is mentioned in notes 14 and 17, it is not reflected as a separate line in the statement of changes in equity).</t>
+          <t>The financial statements include an income statement, statement of financial position, statement of changes in equity, and notes, but no cash flow statement. The company claims the exemption as a qualifying entity (note 2.1), so its absence may be permitted. However, whether all other required components are present depends on whether the exemption is validly taken.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - MISSING</t>
+          <t>Disclosure - verify present</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>FRS102 6.2</t>
+          <t>FRS102 3.21</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -715,12 +715,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: the effects of changes in accounting policies and corrections of material errors recognised in the period</t>
+          <t>Could not confirm this required disclosure - verify: Present each financial statement within a complete set of financial statements with equal prominence.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>The statement of changes in equity does not include a separate row for effects of changes in accounting policies or corrections of material errors. The restatement of 2023 intercompany balances is disclosed only in notes 14 and 17, not in the statement of changes in equity.</t>
+          <t>The financial statements are all included in the same document but there is no explicit statement that each is presented with equal prominence; this is a presentation matter that cannot be fully assessed from narrative text alone.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -741,22 +741,22 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>FRS102 9.8</t>
+          <t>FRS102 5.7E</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Statutory (materiality-blind)</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Could not confirm this required disclosure - verify: Do not exclude a subsidiary from consolidation solely because its business activities are dissimilar to those of other entities within the group.</t>
+          <t>Could not confirm this required disclosure - verify: Disclose on the face of the income statement (or statement of comprehensive income if presented) an amount comprising the total of [the items required by paragraph 5.7E — paragraph text as supplied is truncated and the specific sub-items cannot be determined from the verbatim text provided]</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>The accounts state the company is exempt from preparing consolidated statements under s400 CA 2006 but do not explicitly address the FRS 102 paragraph 9.8 requirement regarding dissimilar activities as a basis for exclusion.</t>
+          <t>The income statement shows turnover, cost of sales, gross profit, administrative expenses, operating loss/profit, interest, and tax. Without knowing the specific sub-items required by paragraph 5.7E (text truncated), it is unclear whether all required line items are present on the face of the income statement.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -777,22 +777,22 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>FRS102 2.11</t>
+          <t>FRS102 6.2</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Statutory (materiality-blind)</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
+          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: the effects of changes in accounting policies and corrections of material errors recognised in the period (this row covers one sub-element of paragraph 6.2; companion rows should address profit or loss, OCI, and investments/dividends/distributions)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>There is no disclosure of any changes in accounting policies or their effects; the accounts state 'The accounting policies have all been applied consistently throughout the year and preceding year.'</t>
+          <t>The statement of changes in equity shows only opening balance, profit/loss for the year, and closing balance. No effects of changes in accounting policies or corrections of material errors are presented as a separate row (the restatement relates to a presentation change in note 14 but is not reflected as a separate line in the SOCE).</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -808,12 +808,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - MISSING</t>
+          <t>Disclosure - verify present</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>FRS102 2.11</t>
+          <t>FRS102 6.2</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -823,12 +823,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
+          <t>Could not confirm this required disclosure - verify: Present in the statement of changes in equity: (1) profit or loss for the reporting period; (2) other comprehensive income for the period; (3) effects of changes in accounting policies and corrections of material errors recognised in the period; and (4) amounts of investments by, and dividends and other distributions to, equity investors during the period</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>There is no disclosure of any changes in accounting policies or their effects; the accounts state 'The accounting policies have all been applied consistently throughout the year and preceding year.'</t>
+          <t>The statement of changes in equity shows profit or loss for the period but does not explicitly show OCI, effects of accounting policy changes/error corrections, or investments/dividends/distributions as separate line items. OCI is noted as nil in the income statement, and no dividends appear to have been paid, but the statement does not present all four elements explicitly.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -844,27 +844,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - verify present</t>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>FRS102/CA06 going_concern_fronthalf</t>
+          <t>FRS102 6.2</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Statutory (materiality-blind)</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Could not confirm this required disclosure - verify: The directors' report or strategic report should address the going concern basis of preparation.</t>
+          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: the effects of changes in accounting policies and corrections of material errors recognised in the period</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>The auditor's report states 'the directors' use of the going concern basis of accounting in the preparation of the financial statements is appropriate' but there is no explicit going concern statement by the directors themselves in the directors' report or strategic report in the narrative provided.</t>
+          <t>The statement of changes in equity does not include a separate line for effects of changes in accounting policies or corrections of material errors. The 2023 restatement (note 14) is not reflected as a separate adjustment row in the SOCE.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -878,27 +878,31 @@
       <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Numerical - cast</t>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>balance_sheet:total_current_assets</t>
+          <t>FRS102 6.2</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Standard - immaterial candidate</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>'(line 8)' (prior) does not cast: components sum to 10367978, statement shows 10367972 (tolerance 2). PROBABLE OCR MISREAD (single digit), candidates by ascending OCR confidence (most likely the first): 'Debtors' read 7,888,837 but casting implies 7,888,831 [OCR confidence 0.962]; 'Cash at bank and in hand' read 2,130,087 but casting implies 2,130,081 [OCR confidence 0.993]; 'Stocks' read 349,054 but casting implies 349,048 [OCR confidence 0.996]; the total '(line 8)' read 10,367,972 but components imply 10,367,978 — re-read/verify before treating as a finding.</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr"/>
+          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: amounts of investments by, and dividends and other distributions to, equity investors during the period</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>The statement of changes in equity shows no row for investments by, or dividends and other distributions to, equity investors. No dividends are disclosed anywhere in the financial statements.</t>
+        </is>
+      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
           <t>open</t>
@@ -910,27 +914,31 @@
       <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Numerical - cross_reference</t>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>note 14 total casts to Debtors on the balance_sheet</t>
+          <t>FRS102 33.10</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Standard - immaterial candidate</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>note 14 total casts to Debtors on the balance_sheet (prior): Total=7888831 != Debtors=7888837 (tolerance 1). PROBABLE OCR MISREAD (single digit) — the two figures differ by a digit; re-read/verify against the document before treating as a finding.</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr"/>
+          <t>Required disclosure not found in the accounts: Disclose the information required by paragraph 33.9 separately for each of the following categories of related party: (a) entities with control, joint control or significant influence over the entity; (b) subsidiaries; (c) associates; (d) joint ventures in which the entity is a venturer; (e) key management personnel; (f) other related parties.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Note 24 states the company has taken the exemption from disclosing intra-group transactions. No disclosure is made separately for each category of related party (e.g. key management personnel, entities with control/significant influence). Key management personnel compensation is also explicitly exempted under note 2.1.</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>open</t>
@@ -942,34 +950,34 @@
       <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Numerical - low_confidence</t>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>balance_sheet:called_up_share_capital</t>
+          <t>FRS102 9.8</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Standard - material</t>
+          <t>Statutory (materiality-blind)</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>'Called up share capital' prior figure 206,541 extracted at low OCR confidence 0.852 — verify against the document</t>
+          <t>Required disclosure not found in the accounts: Do not exclude a subsidiary from consolidation solely because its business activities are dissimilar to those of other entities within the group.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>could not evaluate - confirm</t>
+          <t>The accounts do not address the requirement not to exclude a subsidiary on grounds of dissimilar activities. No discussion of this topic appears anywhere in the financial statements.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>unverified</t>
+          <t>open</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
@@ -978,34 +986,34 @@
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Numerical - low_confidence</t>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>balance_sheet:share_premium_account</t>
+          <t>FRS102 2.11</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Standard - material</t>
+          <t>Statutory (materiality-blind)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>'Share premium account' prior figure 1,093,221 extracted at low OCR confidence 0.836 — verify against the document</t>
+          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>could not evaluate - confirm</t>
+          <t>The accounts do not explicitly disclose any changes in accounting policies or their effects. The restatement of group undertaking balances (note 14) is described as a presentation change, but no formal accounting policy change disclosure with effects is provided.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>unverified</t>
+          <t>open</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
@@ -1014,14 +1022,14 @@
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Judgment - judgment</t>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>FRS102 10.21</t>
+          <t>FRS102 2.11</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1031,10 +1039,14 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>The 2023 comparatives in the statement of financial position and notes 14 and 17 are labelled 'as restated', arising from the netting of intercompany balances under a Multilateral Netting Deed. Note 14 explains the nature of the presentational change and quantifies the gross amounts offset (amounts owed to group undertakings of £26.5m offset against £28.8m owed by group undertakings). However, the accounts treat this as a restatement of comparatives without disclosing whether this constitutes correction of a prior period error or a change in accounting policy, and critically the statement of changes in equity shows no adjustment to opening equity and the income statement comparatives carry no 'as restated' label, meaning the line-by-line effect of the correction on each affected financial statement line and the cumulative effect on opening equity are not disclosed as required. FRS 102 paragraph 10.21 requires that a material prior period error be corrected by restating the comparative amounts and disclosing the nature of the error and the amount of the correction for each financial statement line item affected. (confidence 0.75)</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr"/>
+          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Same as above — no disclosure of changes in accounting policies and their effects is made in the financial statements.</t>
+        </is>
+      </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
           <t>open</t>
@@ -1048,22 +1060,22 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Judgment - judgment</t>
+          <t>Numerical - cast</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>FRS102 29.6</t>
+          <t>balance_sheet:total_current_assets</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Standard - material</t>
+          <t>Standard - immaterial candidate</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>The company has recognised a deferred tax asset of £41,970 at 31 December 2024, of which £41,306 relates to tax losses carried forward. The company reported an operating loss and EBITDA loss in 2024, and the accounts note difficult trading conditions and reduced profitability. There is no explicit evidence provided in the notes or accounting policy disclosures demonstrating that recovery of the tax loss element against future taxable profits is probable. The accounting policy (note 2.13) correctly limits recognition to amounts probable of recovery, but note 15 and the surrounding narrative provide no forward-looking assessment or probability analysis to support the recoverability of the £41,306 loss-related deferred tax asset, creating doubt as to whether the recognition threshold has been met. (confidence 0.72)</t>
+          <t>'(line 8)' (prior) does not cast: components sum to 10367978, statement shows 10367972 (tolerance 2). PROBABLE OCR MISREAD (single digit), candidates by ascending OCR confidence (most likely the first): 'Debtors' read 7,888,837 but casting implies 7,888,831 [OCR confidence 0.962]; 'Cash at bank and in hand' read 2,130,087 but casting implies 2,130,081 [OCR confidence 0.993]; 'Stocks' read 349,054 but casting implies 349,048 [OCR confidence 0.996]; the total '(line 8)' read 10,367,972 but components imply 10,367,978 — re-read/verify before treating as a finding.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
@@ -1074,10 +1086,210 @@
       </c>
       <c r="H14" s="4" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Numerical - cross_reference</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>note 14 total casts to Debtors on the balance_sheet</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Standard - immaterial candidate</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>note 14 total casts to Debtors on the balance_sheet (prior): Total=7888831 != Debtors=7888837 (tolerance 1). PROBABLE OCR MISREAD (single digit) — the two figures differ by a digit; re-read/verify against the document before treating as a finding.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Numerical - low_confidence</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>balance_sheet:called_up_share_capital</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Standard - material</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>'Called up share capital' prior figure 206,541 extracted at low OCR confidence 0.852 — verify against the document</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>could not evaluate - confirm</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Numerical - low_confidence</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>balance_sheet:share_premium_account</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Standard - material</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>'Share premium account' prior figure 1,093,221 extracted at low OCR confidence 0.836 — verify against the document</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>could not evaluate - confirm</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Judgment - judgment</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>FRS102 1AC.3</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Standard - material</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Policy 2.16 (Share capital) states that 'incremental costs directly attributable to the issue of new ordinary shares or options are shown in equity as a deduction, net of tax, from the proceeds.' The statement of changes in equity and share capital note show that the share capital and share premium account were unchanged in both 2024 and 2023 (no new shares were issued in either year), and there is no indication of any share issue costs in either period. The policy relating to costs of issuing new shares is therefore irrelevant boilerplate in both years and does not reflect any actual transaction of this entity. Including inapplicable policies without entity-specific tailoring reduces the clarity and understandability of the financial statements for users, contrary to FRS 102's requirement that policies disclosed should be those actually adopted by the entity in determining the amounts shown. (confidence 0.72)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Judgment - judgment</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>FRS102 10.21</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Standard - material</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>The 2023 comparatives in the statement of financial position and notes 14 and 17 are labelled 'As restated' due to the netting of intercompany balances under the Group's Multilateral Netting Deed. Note 14 explains the nature of the reclassification but does not disclose the amount of the correction for each financial statement line affected by the restatement (e.g. the gross amounts removed from creditors and the net effect on the statement of financial position line totals), nor does it confirm whether this is treated as a prior period error under FRS 102 Section 10 or merely a reclassification. The accounts contain no note identifying the nature of the error (omission of netting), the period(s) affected, or the amount of the correction for each line item restated, as required by FRS 102. (confidence 0.78)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Judgment - judgment</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>FRS102 29.6</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Standard - material</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>The accounts recognise a deferred tax asset of £41,970 at 31 December 2024, of which £41,306 relates to tax losses carried forward. The company reported an operating loss of £291,475 and an EBITDA loss of £270,276 in 2024, following a significant decline in turnover and gross profit. While the directors express optimism about future recovery, the accounts contain no explicit assessment or disclosure of whether it is probable that sufficient future taxable profits will be available to recover the losses element of the deferred tax asset. Under FRS 102, recognition of a deferred tax asset on tax losses is limited to the extent it is probable they will be recovered against future taxable profits; given the loss-making position and the scale of restructuring, the absence of any recoverability assessment or disclosure creates a risk that the asset is overstated. (confidence 0.72)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H20"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"accept,reject,amend,immaterial"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1091,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1125,17 +1337,17 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>applies_hedge_accounting_section12</t>
+          <t>not_going_concern</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Does the entity apply hedge accounting under Section 12 (Financial Instruments) of FRS 102?</t>
+          <t>Is there any doubt about the company's ability to continue operating as a going concern over the next 12 months, or have you identified circumstances that suggest it may not be able to pay its debts as they fall due?</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>FRS102 12.26, FRS102 12.27, FRS102 12.29, FRS102 12.29A</t>
+          <t>FRS102 3.9, FRS102 32.7B</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr"/>
@@ -1143,17 +1355,17 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>applies_section12</t>
+          <t>has_going_concern_material_uncertainties</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Does the entity have financial instruments in scope of Section 12 (Financial Instruments) of FRS 102?</t>
+          <t>Are there any significant events or conditions that create material uncertainty about whether the company will remain a going concern, even though you currently believe it will?</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>FRS102 12.26, FRS102 12.29, FRS102 12.29A</t>
+          <t>FRS102 3.9</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr"/>
@@ -1161,17 +1373,17 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>has_heritage_assets</t>
+          <t>has_key_estimation_uncertainties</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Does the entity hold any heritage assets as defined by FRS 102?</t>
+          <t>Are there any areas of the financial statements where you've had to make judgements or estimates that are particularly sensitive to changes in assumptions, or where outcomes could significantly differ from what you've recorded?</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>FRS102 34.52, FRS102 34.55, FRS102 34.63</t>
+          <t>FRS102 8.7</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr"/>
@@ -1179,17 +1391,17 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>has_non_trading_non_derivative_section12_instruments</t>
+          <t>has_material_prior_period_error</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Does the entity hold non-trading, non-derivative financial instruments within the scope of Section 12?</t>
+          <t>Have you discovered any errors in amounts reported in the previous year's financial statements that were material enough to require correction, rather than just being caught this year and dealt with prospectively?</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>FRS102 11.42, FRS102 12.26</t>
+          <t>FRS102 10.21</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr"/>
@@ -1197,17 +1409,17 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>has_probable_contingent_assets</t>
+          <t>dividend_recommended</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Does the entity have contingent assets that are probable of occurring?</t>
+          <t>Did the directors recommend or pay a dividend for the year?</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>FRS102 21.16, FRS102 21.17</t>
+          <t>CA06 s416(3)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
@@ -1215,398 +1427,20 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>has_termination_benefits</t>
+          <t>average_employees_gt_250</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Has the entity incurred or committed to termination benefits for employees during the period?</t>
+          <t>Did the company employ on average more than 250 people during the year?</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>FRS102 28.43, FRS102 28.44</t>
+          <t>SI2008/410 Sch7 para10-11</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>has_transferred_financial_assets_not_derecognised</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Does the entity have transferred financial assets that have not been derecognised from the statement of financial position?</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 11.42, FRS102 11.45</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>has_unremedied_loan_breach_or_default</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Does the entity have any loan facility breaches or defaults that remain unremedied at the reporting date?</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 11.42, FRS102 11.47</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>measures_group_rented_investment_property_at_cost</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Does the group measure rented investment property at cost rather than fair value?</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 17.30A, FRS102 17.31A</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>uses_equity_method_for_associates</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Does the entity use the equity method to account for investments in associates?</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 14.12, FRS102 14.14</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>uses_indirect_method_cash_flow</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Does the entity prepare its cash flow statement using the indirect method?</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 7.8, FRS102 7.9</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>additional_soci_line_items_relevant</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Are there additional line items relevant to the entity's statement of comprehensive income beyond the standard items?</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 5.9</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>additional_sofp_line_items_relevant</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Are there additional line items relevant to the entity's statement of financial position beyond the standard items?</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 4.3</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>applicable_sorp_exists</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Is there an applicable Statement of Recommended Practice (SORP) that applies to the entity's activities?</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 1.7A</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>associate_equity_method_with_quoted_price</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Does an associate accounted for under the equity method have a quoted market price available?</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 14.12</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>associate_has_discontinued_operations</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Does any associate have discontinued operations during or before the reporting period?</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 14.14</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>capitalises_borrowing_costs</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Does the entity capitalise any borrowing costs as part of the cost of qualifying assets?</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 25.3A</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>cash_and_cash_equivalents_sofp_matches_scf</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Does the cash and cash equivalents balance in the statement of financial position reconcile to the opening balance in the statement of cash flows?</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 7.20</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>debtors_after_one_year_material_to_net_current_assets</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Are debtors due after more than one year material in relation to the entity's net current assets?</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 4.4A</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>financial_instrument_information_is_material</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Is the disclosure of financial instrument information material to the financial statements as a whole?</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 11.42</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>future_period_effect_of_estimate_change_practicable</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Is it practicable to estimate the effect of accounting estimate changes in future periods?</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 10.18</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>has_accounting_estimate_changes</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Has the entity made any changes to accounting estimates during the reporting period?</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 10.18</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>has_any_discontinued_operations_by_end_of_latest_reporting_period</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Does the entity have any discontinued operations that existed by the end of the latest reporting period?</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 5.7F</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>has_artificial_or_no_substance_exchange_transaction</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Has the entity entered into any exchange transactions that lack commercial substance or are artificial in nature?</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 9.32</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>has_binding_sale_agreement_for_major_disposal</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Does the entity have a binding agreement in place for the sale of a major asset or disposal group?</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 4.14</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>dividend_recommended</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Does the directors' report state the dividend the directors recommend (or that none is recommended)? CA06 s416(3) requires this to be stated.</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>CA06 s416(3)</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>average_employees_gt_250</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Did the company employ on average more than 250 people in the year? If so, the directors' report must include an employee-engagement statement (Sch 7 para 11) and a statement of policy on the employment of disabled persons (Sch 7 para 10). Both are not required below 250 employees.</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>SI2008/410 Sch7 para10-11</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refresh FC findings cache: 17 -> 12, false positives cleared
With the gating + OCR second-loop in place, the FC register no longer shows the
rule-quality false positives Phil rejected: 3.6 (departure), 9.8 (consolidation),
the 3.17 complete-set components, 3.21, the 6.2 SOCE rows, and the 1AC.3 boilerplate
are all gone. The prior-year current-assets cast is now reported as a "suspected
OCR misread - verify" rather than a casting error. What remains is genuine: two
judgement confirms (10.21 restatement, 29.6 deferred tax), the known OCR/low-
confidence numerics, two real missing disclosures (33.10, 2.11) and a few softer
"verify" prompts (5.7C/5.9B/21.14/29.20).
</commit_message>
<xml_diff>
--- a/build/summaries/FC-register.xlsx
+++ b/build/summaries/FC-register.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Questions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues register'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues register'!$A$1:$H$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,21 +511,21 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Required disclosures missing: 8</t>
+          <t>Required disclosures missing: 3</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Disclosures to verify present: 4</t>
+          <t>Disclosures to verify present: 5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Numerical findings: 5 (2 could not be evaluated)</t>
+          <t>Numerical findings: 4 (2 could not be evaluated)</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Checklist outcomes: not_applicable=284, encouraged=2, applicable=72, undetermined=7</t>
+          <t>Checklist outcomes: not_applicable=298, encouraged=2, applicable=57, undetermined=7</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -628,12 +628,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - MISSING</t>
+          <t>Disclosure - verify present</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>FRS102 3.6</t>
+          <t>FRS102 5.7C</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -643,12 +643,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Where an entity departed from a requirement of FRS 102 or applicable legislation in a prior period and that departure affects amounts recognised in the current period, disclose the information required by paragraph 3.5(c).</t>
+          <t>Could not confirm this required disclosure - verify: The statement of comprehensive income shall begin with profit or loss as its first line and shall display, as a minimum, line items presenting the amounts described in paragraphs 5.5A and 5.6(b) for the period.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>There is no disclosure of any prior period departure from FRS 102 or applicable legislation that affects amounts in the current period, beyond the restatement of group undertaking balances which is explained in note 14 but not framed as a departure from a requirement.</t>
+          <t>The company has not presented a separate statement of comprehensive income (as noted: 'no statement of other comprehensive income has been presented'). The income statement ends with profit/loss for the year. It is unclear whether a combined statement of comprehensive income beginning with profit or loss was required given no OCI items exist.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>FRS102 3.17</t>
+          <t>FRS102 5.7E</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -679,12 +679,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Could not confirm this required disclosure - verify: A complete set of financial statements shall include all of the required components as listed in paragraph 3.17 (e.g. a statement of financial position, a statement of comprehensive income or equivalent, a cash flow statement, a statement of changes in equity, and notes).</t>
+          <t>Could not confirm this required disclosure - verify: Disclose on the face of the income statement (or statement of comprehensive income if presented) an amount comprising the total of [the items required by paragraph 5.7E — paragraph text as supplied is truncated and the specific sub-items cannot be determined from the verbatim text provided]</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>The financial statements include an income statement, statement of financial position, statement of changes in equity, and notes, but no cash flow statement. The company claims the exemption as a qualifying entity (note 2.1), so its absence may be permitted. However, whether all other required components are present depends on whether the exemption is validly taken.</t>
+          <t>Paragraph 5.7E requirements cannot be fully assessed as the specific sub-items required are noted as truncated in the question. The income statement does present various line items including one-off administrative expenses separately, but without knowing the exact sub-items of 5.7E, this cannot be confirmed.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>FRS102 3.21</t>
+          <t>FRS102 5.9B</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -715,12 +715,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Could not confirm this required disclosure - verify: Present each financial statement within a complete set of financial statements with equal prominence.</t>
+          <t>Could not confirm this required disclosure - verify: If operating profit is disclosed, profits or losses on the disposal of a discontinued operation shall be excluded from operating profit.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>The financial statements are all included in the same document but there is no explicit statement that each is presented with equal prominence; this is a presentation matter that cannot be fully assessed from narrative text alone.</t>
+          <t>The accounts do not appear to have any discontinued operations, so this requirement is not triggered. There is no evidence of a discontinued operation being excluded or included in operating profit.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>FRS102 5.7E</t>
+          <t>FRS102 21.14</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -751,12 +751,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Could not confirm this required disclosure - verify: Disclose on the face of the income statement (or statement of comprehensive income if presented) an amount comprising the total of [the items required by paragraph 5.7E — paragraph text as supplied is truncated and the specific sub-items cannot be determined from the verbatim text provided]</t>
+          <t>Could not confirm this required disclosure - verify: For each class of provision, disclose the following (the paragraph head; sub-items are listed in the full 21.14 text and include: the carrying amount at the beginning and end of the period; additional provisions made in the period, including increases to existing provisions; amounts used during the period; unused amounts reversed during the period; and the unwinding of any discount or change in the discount rate).</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>The income statement shows turnover, cost of sales, gross profit, administrative expenses, operating loss/profit, interest, and tax. Without knowing the specific sub-items required by paragraph 5.7E (text truncated), it is unclear whether all required line items are present on the face of the income statement.</t>
+          <t>Note 26 discloses the carrying amount at end of period (£99,561) and additions charged to profit or loss (£99,561), but does not separately disclose opening balance (nil implied), amounts used, amounts reversed, or unwinding of discount as required by 21.14.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - MISSING</t>
+          <t>Disclosure - verify present</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>FRS102 6.2</t>
+          <t>FRS102 29.20</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -787,12 +787,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: the effects of changes in accounting policies and corrections of material errors recognised in the period (this row covers one sub-element of paragraph 6.2; companion rows should address profit or loss, OCI, and investments/dividends/distributions)</t>
+          <t>Could not confirm this required disclosure - verify: Expenses shown in profit or loss shall exclude recoverable VAT and other similar recoverable sales taxes.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>The statement of changes in equity shows only opening balance, profit/loss for the year, and closing balance. No effects of changes in accounting policies or corrections of material errors are presented as a separate row (the restatement relates to a presentation change in note 14 but is not reflected as a separate line in the SOCE).</t>
+          <t>The accounts do not explicitly state that expenses exclude recoverable VAT; while this is implied by normal accounting practice, no explicit disclosure is made.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -808,12 +808,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Disclosure - verify present</t>
+          <t>Disclosure - MISSING</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>FRS102 6.2</t>
+          <t>FRS102 33.10</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -823,12 +823,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Could not confirm this required disclosure - verify: Present in the statement of changes in equity: (1) profit or loss for the reporting period; (2) other comprehensive income for the period; (3) effects of changes in accounting policies and corrections of material errors recognised in the period; and (4) amounts of investments by, and dividends and other distributions to, equity investors during the period</t>
+          <t>Required disclosure not found in the accounts: Disclose the information required by paragraph 33.9 separately for each of the following categories of related party: (a) entities with control, joint control or significant influence over the entity; (b) subsidiaries; (c) associates; (d) joint ventures in which the entity is a venturer; (e) key management personnel; (f) other related parties.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>The statement of changes in equity shows profit or loss for the period but does not explicitly show OCI, effects of accounting policy changes/error corrections, or investments/dividends/distributions as separate line items. OCI is noted as nil in the income statement, and no dividends appear to have been paid, but the statement does not present all four elements explicitly.</t>
+          <t>Note 24 takes the FRS 102 33.1A exemption for intra-group transactions. There is no disclosure of transactions with key management personnel or other related party categories separately as required by 33.10.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -849,22 +849,22 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>FRS102 6.2</t>
+          <t>FRS102 2.11</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Standard - material</t>
+          <t>Statutory (materiality-blind)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: the effects of changes in accounting policies and corrections of material errors recognised in the period</t>
+          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>The statement of changes in equity does not include a separate line for effects of changes in accounting policies or corrections of material errors. The 2023 restatement (note 14) is not reflected as a separate adjustment row in the SOCE.</t>
+          <t>There is no disclosure of any changes in accounting policies or their effects. The accounts state 'The accounting policies have all been applied consistently throughout the year and preceding year' but no specific change disclosure is made (none appears to have occurred).</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>FRS102 6.2</t>
+          <t>FRS102 2.11</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -895,12 +895,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Present in the statement of changes in equity: amounts of investments by, and dividends and other distributions to, equity investors during the period</t>
+          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>The statement of changes in equity shows no row for investments by, or dividends and other distributions to, equity investors. No dividends are disclosed anywhere in the financial statements.</t>
+          <t>As with index 18, no changes in accounting policies are disclosed or described. The accounts confirm consistent application of policies with no changes noted.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -914,31 +914,27 @@
       <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Disclosure - MISSING</t>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Numerical - cast</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>FRS102 33.10</t>
+          <t>balance_sheet:total_current_assets</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Standard - material</t>
+          <t>Standard - immaterial candidate</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Disclose the information required by paragraph 33.9 separately for each of the following categories of related party: (a) entities with control, joint control or significant influence over the entity; (b) subsidiaries; (c) associates; (d) joint ventures in which the entity is a venturer; (e) key management personnel; (f) other related parties.</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Note 24 states the company has taken the exemption from disclosing intra-group transactions. No disclosure is made separately for each category of related party (e.g. key management personnel, entities with control/significant influence). Key management personnel compensation is also explicitly exempted under note 2.1.</t>
-        </is>
-      </c>
+          <t>'(line 8)' (prior) suspected OCR misread: components sum to 10367978 but the statement shows 10367972; the corrected value is corroborated elsewhere in the document — verify the figure. PROBABLE OCR MISREAD (single digit), candidates by ascending OCR confidence (most likely the first): 'Debtors' read 7,888,837 but casting implies 7,888,831 [OCR confidence 0.962] — corroborated elsewhere in the document; 'Cash at bank and in hand' read 2,130,087 but casting implies 2,130,081 [OCR confidence 0.993]; 'Stocks' read 349,054 but casting implies 349,048 [OCR confidence 0.996]; the total '(line 8)' read 10,367,972 but components imply 10,367,978 — re-read/verify before treating as a finding.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>open</t>
@@ -950,31 +946,27 @@
       <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Disclosure - MISSING</t>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Numerical - cross_reference</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>FRS102 9.8</t>
+          <t>note 14 total casts to Debtors on the balance_sheet</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Statutory (materiality-blind)</t>
+          <t>Standard - immaterial candidate</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Do not exclude a subsidiary from consolidation solely because its business activities are dissimilar to those of other entities within the group.</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>The accounts do not address the requirement not to exclude a subsidiary on grounds of dissimilar activities. No discussion of this topic appears anywhere in the financial statements.</t>
-        </is>
-      </c>
+          <t>note 14 total casts to Debtors on the balance_sheet (prior): Total=7888831 != Debtors=7888837 (tolerance 1). PROBABLE OCR MISREAD (single digit) — the two figures differ by a digit; re-read/verify against the document before treating as a finding.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
           <t>open</t>
@@ -986,34 +978,34 @@
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Disclosure - MISSING</t>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Numerical - low_confidence</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>FRS102 2.11</t>
+          <t>balance_sheet:called_up_share_capital</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Statutory (materiality-blind)</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
+          <t>'Called up share capital' prior figure 206,541 extracted at low OCR confidence 0.852 — verify against the document</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>The accounts do not explicitly disclose any changes in accounting policies or their effects. The restatement of group undertaking balances (note 14) is described as a presentation change, but no formal accounting policy change disclosure with effects is provided.</t>
+          <t>could not evaluate - confirm</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>unverified</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
@@ -1022,14 +1014,14 @@
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Disclosure - MISSING</t>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Numerical - low_confidence</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>FRS102 2.11</t>
+          <t>balance_sheet:share_premium_account</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1039,17 +1031,17 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Required disclosure not found in the accounts: Disclose any changes in accounting policies and the effects of such changes</t>
+          <t>'Share premium account' prior figure 1,093,221 extracted at low OCR confidence 0.836 — verify against the document</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Same as above — no disclosure of changes in accounting policies and their effects is made in the financial statements.</t>
+          <t>could not evaluate - confirm</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>unverified</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
@@ -1060,22 +1052,22 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Numerical - cast</t>
+          <t>Judgment - judgment</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>balance_sheet:total_current_assets</t>
+          <t>FRS102 10.21</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Standard - immaterial candidate</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>'(line 8)' (prior) does not cast: components sum to 10367978, statement shows 10367972 (tolerance 2). PROBABLE OCR MISREAD (single digit), candidates by ascending OCR confidence (most likely the first): 'Debtors' read 7,888,837 but casting implies 7,888,831 [OCR confidence 0.962]; 'Cash at bank and in hand' read 2,130,087 but casting implies 2,130,081 [OCR confidence 0.993]; 'Stocks' read 349,054 but casting implies 349,048 [OCR confidence 0.996]; the total '(line 8)' read 10,367,972 but components imply 10,367,978 — re-read/verify before treating as a finding.</t>
+          <t>The 2023 comparative figures in the statement of financial position and notes 14 and 17 are labelled 'As restated', reflecting the netting of intercompany balances under the Group's Multilateral Netting Deed (offsetting £26.5m owed to group undertakings against £28.8m owed by group undertakings). Although note 14 briefly describes the mechanical restatement, the accounts do not disclose the nature of the prior period error (i.e. whether this is a correction of a misstatement or a change in accounting policy), do not quantify the correction on each individual line of the statement of financial position affected (e.g. the gross reduction to both debtors and creditors is stated only in note 14 but not for the statement of financial position line totals or net assets), and provide no explanation in a dedicated prior period adjustment note as required. FRS 102 paragraph 10.21 requires an entity correcting a material prior period error to disclose the nature of the error and the amount of the correction for each financial statement line item affected. (confidence 0.78)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
@@ -1092,22 +1084,22 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Numerical - cross_reference</t>
+          <t>Judgment - judgment</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>note 14 total casts to Debtors on the balance_sheet</t>
+          <t>FRS102 29.6</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Standard - immaterial candidate</t>
+          <t>Standard - material</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>note 14 total casts to Debtors on the balance_sheet (prior): Total=7888831 != Debtors=7888837 (tolerance 1). PROBABLE OCR MISREAD (single digit) — the two figures differ by a digit; re-read/verify against the document before treating as a finding.</t>
+          <t>The company recognises a deferred tax asset of £41,970 at 31 December 2024, of which £41,306 relates to tax losses carried forward. The company reported an operating loss for 2024 and has experienced declining revenues and profitability over multiple years. While the directors express optimism about future trading, no explicit evidence or disclosure is provided in the notes demonstrating that it is probable these tax losses will be recovered against future taxable profits. FRS 102 requires that recognition of deferred tax assets on tax losses is limited to the extent recovery is probable, yet the accounts contain no assessment of the sufficiency or timing of anticipated future taxable profits to support recoverability of the loss-related deferred tax asset. (confidence 0.72)</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
@@ -1118,178 +1110,10 @@
       </c>
       <c r="H15" s="4" t="inlineStr"/>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Numerical - low_confidence</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>balance_sheet:called_up_share_capital</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Standard - material</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>'Called up share capital' prior figure 206,541 extracted at low OCR confidence 0.852 — verify against the document</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>could not evaluate - confirm</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Numerical - low_confidence</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>balance_sheet:share_premium_account</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Standard - material</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>'Share premium account' prior figure 1,093,221 extracted at low OCR confidence 0.836 — verify against the document</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>could not evaluate - confirm</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Judgment - judgment</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 1AC.3</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Standard - material</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Policy 2.16 (Share capital) states that 'incremental costs directly attributable to the issue of new ordinary shares or options are shown in equity as a deduction, net of tax, from the proceeds.' The statement of changes in equity and share capital note show that the share capital and share premium account were unchanged in both 2024 and 2023 (no new shares were issued in either year), and there is no indication of any share issue costs in either period. The policy relating to costs of issuing new shares is therefore irrelevant boilerplate in both years and does not reflect any actual transaction of this entity. Including inapplicable policies without entity-specific tailoring reduces the clarity and understandability of the financial statements for users, contrary to FRS 102's requirement that policies disclosed should be those actually adopted by the entity in determining the amounts shown. (confidence 0.72)</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Judgment - judgment</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 10.21</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Standard - material</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>The 2023 comparatives in the statement of financial position and notes 14 and 17 are labelled 'As restated' due to the netting of intercompany balances under the Group's Multilateral Netting Deed. Note 14 explains the nature of the reclassification but does not disclose the amount of the correction for each financial statement line affected by the restatement (e.g. the gross amounts removed from creditors and the net effect on the statement of financial position line totals), nor does it confirm whether this is treated as a prior period error under FRS 102 Section 10 or merely a reclassification. The accounts contain no note identifying the nature of the error (omission of netting), the period(s) affected, or the amount of the correction for each line item restated, as required by FRS 102. (confidence 0.78)</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Judgment - judgment</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>FRS102 29.6</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Standard - material</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>The accounts recognise a deferred tax asset of £41,970 at 31 December 2024, of which £41,306 relates to tax losses carried forward. The company reported an operating loss of £291,475 and an EBITDA loss of £270,276 in 2024, following a significant decline in turnover and gross profit. While the directors express optimism about future recovery, the accounts contain no explicit assessment or disclosure of whether it is probable that sufficient future taxable profits will be available to recover the losses element of the deferred tax asset. Under FRS 102, recognition of a deferred tax asset on tax losses is limited to the extent it is probable they will be recovered against future taxable profits; given the loss-making position and the scale of restructuring, the absence of any recoverability assessment or disclosure creates a risk that the asset is overstated. (confidence 0.72)</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H15"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"accept,reject,amend,immaterial"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1342,7 +1166,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Is there any doubt about the company's ability to continue operating as a going concern over the next 12 months, or have you identified circumstances that suggest it may not be able to pay its debts as they fall due?</t>
+          <t>Is the company expected to continue operating as a going concern over the next twelve months, or are there circumstances that mean it might not?</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -1360,7 +1184,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Are there any significant events or conditions that create material uncertainty about whether the company will remain a going concern, even though you currently believe it will?</t>
+          <t>Are there any significant uncertainties about whether the company will be able to continue as a going concern that management has identified?</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1378,7 +1202,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Are there any areas of the financial statements where you've had to make judgements or estimates that are particularly sensitive to changes in assumptions, or where outcomes could significantly differ from what you've recorded?</t>
+          <t>Are there any areas in the financial statements where the outcome is particularly uncertain and depends heavily on management's judgement or assumptions?</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1396,7 +1220,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Have you discovered any errors in amounts reported in the previous year's financial statements that were material enough to require correction, rather than just being caught this year and dealt with prospectively?</t>
+          <t>Have you identified any errors in the prior year financial statements that were material enough to require correction or disclosure?</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">

</xml_diff>